<commit_message>
added playwright whatsapp scripts
</commit_message>
<xml_diff>
--- a/contacts.xlsx
+++ b/contacts.xlsx
@@ -20,33 +20,15 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
   <si>
     <t xml:space="preserve">Phone</t>
   </si>
   <si>
-    <t xml:space="preserve">Name</t>
+    <t xml:space="preserve">status</t>
   </si>
   <si>
-    <t xml:space="preserve">State</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Template Name</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Enquiry From</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kasturi Aich</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kolkata</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LAVANYA_ENGLISH</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Trade India</t>
+    <t xml:space="preserve">sent_at</t>
   </si>
 </sst>
 </file>
@@ -278,245 +260,394 @@
       <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="2" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="2" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+    </row>
+    <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="n">
         <v>7503085792</v>
       </c>
-      <c r="B2" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="C2" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="D2" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="E2" s="3" t="s">
-        <v>8</v>
-      </c>
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D3" s="2"/>
-      <c r="E3" s="2"/>
+      <c r="A3" s="1"/>
+      <c r="B3" s="1"/>
+      <c r="C3" s="1"/>
+      <c r="D3" s="3"/>
+      <c r="E3" s="3"/>
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D4" s="2"/>
-      <c r="E4" s="2"/>
+      <c r="A4" s="1"/>
+      <c r="B4" s="1"/>
+      <c r="C4" s="1"/>
+      <c r="D4" s="3"/>
+      <c r="E4" s="3"/>
     </row>
     <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D5" s="2"/>
-      <c r="E5" s="2"/>
+      <c r="A5" s="1"/>
+      <c r="B5" s="1"/>
+      <c r="C5" s="1"/>
+      <c r="D5" s="3"/>
+      <c r="E5" s="3"/>
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D6" s="2"/>
-      <c r="E6" s="2"/>
+      <c r="A6" s="1"/>
+      <c r="B6" s="1"/>
+      <c r="C6" s="1"/>
+      <c r="D6" s="3"/>
+      <c r="E6" s="3"/>
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D7" s="2"/>
-      <c r="E7" s="2"/>
+      <c r="A7" s="1"/>
+      <c r="B7" s="1"/>
+      <c r="C7" s="1"/>
+      <c r="D7" s="3"/>
+      <c r="E7" s="3"/>
     </row>
     <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D8" s="2"/>
-      <c r="E8" s="2"/>
+      <c r="A8" s="1"/>
+      <c r="B8" s="1"/>
+      <c r="C8" s="1"/>
+      <c r="D8" s="3"/>
+      <c r="E8" s="3"/>
     </row>
     <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D9" s="2"/>
-      <c r="E9" s="2"/>
+      <c r="A9" s="1"/>
+      <c r="B9" s="1"/>
+      <c r="C9" s="1"/>
+      <c r="D9" s="3"/>
+      <c r="E9" s="3"/>
     </row>
     <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D10" s="2"/>
-      <c r="E10" s="2"/>
+      <c r="A10" s="1"/>
+      <c r="B10" s="1"/>
+      <c r="C10" s="1"/>
+      <c r="D10" s="3"/>
+      <c r="E10" s="3"/>
     </row>
     <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D11" s="2"/>
-      <c r="E11" s="2"/>
+      <c r="A11" s="1"/>
+      <c r="B11" s="1"/>
+      <c r="C11" s="1"/>
+      <c r="D11" s="3"/>
+      <c r="E11" s="3"/>
     </row>
     <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D12" s="2"/>
-      <c r="E12" s="2"/>
+      <c r="A12" s="1"/>
+      <c r="B12" s="1"/>
+      <c r="C12" s="1"/>
+      <c r="D12" s="3"/>
+      <c r="E12" s="3"/>
     </row>
     <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D13" s="2"/>
-      <c r="E13" s="2"/>
+      <c r="A13" s="1"/>
+      <c r="B13" s="1"/>
+      <c r="C13" s="1"/>
+      <c r="D13" s="3"/>
+      <c r="E13" s="3"/>
     </row>
     <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D14" s="2"/>
-      <c r="E14" s="2"/>
+      <c r="A14" s="1"/>
+      <c r="B14" s="1"/>
+      <c r="C14" s="1"/>
+      <c r="D14" s="3"/>
+      <c r="E14" s="3"/>
     </row>
     <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D15" s="2"/>
-      <c r="E15" s="2"/>
+      <c r="A15" s="1"/>
+      <c r="B15" s="1"/>
+      <c r="C15" s="1"/>
+      <c r="D15" s="3"/>
+      <c r="E15" s="3"/>
     </row>
     <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D16" s="2"/>
-      <c r="E16" s="2"/>
+      <c r="A16" s="1"/>
+      <c r="B16" s="1"/>
+      <c r="C16" s="1"/>
+      <c r="D16" s="3"/>
+      <c r="E16" s="3"/>
     </row>
     <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D17" s="2"/>
-      <c r="E17" s="2"/>
+      <c r="A17" s="1"/>
+      <c r="B17" s="1"/>
+      <c r="C17" s="1"/>
+      <c r="D17" s="3"/>
+      <c r="E17" s="3"/>
     </row>
     <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D18" s="2"/>
-      <c r="E18" s="2"/>
+      <c r="A18" s="1"/>
+      <c r="B18" s="1"/>
+      <c r="C18" s="1"/>
+      <c r="D18" s="3"/>
+      <c r="E18" s="3"/>
     </row>
     <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D19" s="2"/>
-      <c r="E19" s="2"/>
+      <c r="A19" s="1"/>
+      <c r="B19" s="1"/>
+      <c r="C19" s="1"/>
+      <c r="D19" s="3"/>
+      <c r="E19" s="3"/>
     </row>
     <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D20" s="2"/>
-      <c r="E20" s="2"/>
+      <c r="A20" s="1"/>
+      <c r="B20" s="1"/>
+      <c r="C20" s="1"/>
+      <c r="D20" s="3"/>
+      <c r="E20" s="3"/>
     </row>
     <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D21" s="2"/>
-      <c r="E21" s="2"/>
+      <c r="A21" s="1"/>
+      <c r="B21" s="1"/>
+      <c r="C21" s="1"/>
+      <c r="D21" s="3"/>
+      <c r="E21" s="3"/>
     </row>
     <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D22" s="2"/>
-      <c r="E22" s="2"/>
+      <c r="A22" s="1"/>
+      <c r="B22" s="1"/>
+      <c r="C22" s="1"/>
+      <c r="D22" s="3"/>
+      <c r="E22" s="3"/>
     </row>
     <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D23" s="2"/>
-      <c r="E23" s="2"/>
+      <c r="A23" s="1"/>
+      <c r="B23" s="1"/>
+      <c r="C23" s="1"/>
+      <c r="D23" s="3"/>
+      <c r="E23" s="3"/>
     </row>
     <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D24" s="2"/>
-      <c r="E24" s="2"/>
+      <c r="A24" s="1"/>
+      <c r="B24" s="1"/>
+      <c r="C24" s="1"/>
+      <c r="D24" s="3"/>
+      <c r="E24" s="3"/>
     </row>
     <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D25" s="2"/>
-      <c r="E25" s="2"/>
+      <c r="A25" s="1"/>
+      <c r="B25" s="1"/>
+      <c r="C25" s="1"/>
+      <c r="D25" s="3"/>
+      <c r="E25" s="3"/>
     </row>
     <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D26" s="2"/>
-      <c r="E26" s="2"/>
+      <c r="A26" s="1"/>
+      <c r="B26" s="1"/>
+      <c r="C26" s="1"/>
+      <c r="D26" s="3"/>
+      <c r="E26" s="3"/>
     </row>
     <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D27" s="2"/>
-      <c r="E27" s="2"/>
+      <c r="A27" s="1"/>
+      <c r="B27" s="1"/>
+      <c r="C27" s="1"/>
+      <c r="D27" s="3"/>
+      <c r="E27" s="3"/>
     </row>
     <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D28" s="2"/>
-      <c r="E28" s="2"/>
+      <c r="A28" s="1"/>
+      <c r="B28" s="1"/>
+      <c r="C28" s="1"/>
+      <c r="D28" s="3"/>
+      <c r="E28" s="3"/>
     </row>
     <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D29" s="2"/>
-      <c r="E29" s="2"/>
+      <c r="A29" s="1"/>
+      <c r="B29" s="1"/>
+      <c r="C29" s="1"/>
+      <c r="D29" s="3"/>
+      <c r="E29" s="3"/>
     </row>
     <row r="30" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D30" s="2"/>
-      <c r="E30" s="2"/>
+      <c r="A30" s="1"/>
+      <c r="B30" s="1"/>
+      <c r="C30" s="1"/>
+      <c r="D30" s="3"/>
+      <c r="E30" s="3"/>
     </row>
     <row r="31" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D31" s="2"/>
-      <c r="E31" s="2"/>
+      <c r="A31" s="1"/>
+      <c r="B31" s="1"/>
+      <c r="C31" s="1"/>
+      <c r="D31" s="3"/>
+      <c r="E31" s="3"/>
     </row>
     <row r="32" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D32" s="2"/>
-      <c r="E32" s="2"/>
+      <c r="A32" s="1"/>
+      <c r="B32" s="1"/>
+      <c r="C32" s="1"/>
+      <c r="D32" s="3"/>
+      <c r="E32" s="3"/>
     </row>
     <row r="33" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D33" s="2"/>
-      <c r="E33" s="2"/>
+      <c r="A33" s="1"/>
+      <c r="B33" s="1"/>
+      <c r="C33" s="1"/>
+      <c r="D33" s="3"/>
+      <c r="E33" s="3"/>
     </row>
     <row r="34" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D34" s="2"/>
-      <c r="E34" s="2"/>
+      <c r="A34" s="1"/>
+      <c r="B34" s="1"/>
+      <c r="C34" s="1"/>
+      <c r="D34" s="3"/>
+      <c r="E34" s="3"/>
     </row>
     <row r="35" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D35" s="2"/>
-      <c r="E35" s="2"/>
+      <c r="A35" s="1"/>
+      <c r="B35" s="1"/>
+      <c r="C35" s="1"/>
+      <c r="D35" s="3"/>
+      <c r="E35" s="3"/>
     </row>
     <row r="36" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D36" s="2"/>
-      <c r="E36" s="2"/>
+      <c r="A36" s="1"/>
+      <c r="B36" s="1"/>
+      <c r="C36" s="1"/>
+      <c r="D36" s="3"/>
+      <c r="E36" s="3"/>
     </row>
     <row r="37" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D37" s="2"/>
-      <c r="E37" s="2"/>
+      <c r="A37" s="1"/>
+      <c r="B37" s="1"/>
+      <c r="C37" s="1"/>
+      <c r="D37" s="3"/>
+      <c r="E37" s="3"/>
     </row>
     <row r="38" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D38" s="2"/>
-      <c r="E38" s="2"/>
+      <c r="A38" s="1"/>
+      <c r="B38" s="1"/>
+      <c r="C38" s="1"/>
+      <c r="D38" s="3"/>
+      <c r="E38" s="3"/>
     </row>
     <row r="39" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D39" s="2"/>
-      <c r="E39" s="2"/>
+      <c r="A39" s="1"/>
+      <c r="B39" s="1"/>
+      <c r="C39" s="1"/>
+      <c r="D39" s="3"/>
+      <c r="E39" s="3"/>
     </row>
     <row r="40" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D40" s="2"/>
-      <c r="E40" s="2"/>
+      <c r="A40" s="1"/>
+      <c r="B40" s="1"/>
+      <c r="C40" s="1"/>
+      <c r="D40" s="3"/>
+      <c r="E40" s="3"/>
     </row>
     <row r="41" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D41" s="2"/>
-      <c r="E41" s="2"/>
+      <c r="A41" s="1"/>
+      <c r="B41" s="1"/>
+      <c r="C41" s="1"/>
+      <c r="D41" s="3"/>
+      <c r="E41" s="3"/>
     </row>
     <row r="42" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D42" s="2"/>
-      <c r="E42" s="2"/>
+      <c r="A42" s="1"/>
+      <c r="B42" s="1"/>
+      <c r="C42" s="1"/>
+      <c r="D42" s="3"/>
+      <c r="E42" s="3"/>
     </row>
     <row r="43" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D43" s="2"/>
-      <c r="E43" s="2"/>
+      <c r="A43" s="1"/>
+      <c r="B43" s="1"/>
+      <c r="C43" s="1"/>
+      <c r="D43" s="3"/>
+      <c r="E43" s="3"/>
     </row>
     <row r="44" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D44" s="2"/>
-      <c r="E44" s="2"/>
+      <c r="A44" s="1"/>
+      <c r="B44" s="1"/>
+      <c r="C44" s="1"/>
+      <c r="D44" s="3"/>
+      <c r="E44" s="3"/>
     </row>
     <row r="45" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D45" s="2"/>
-      <c r="E45" s="2"/>
+      <c r="A45" s="1"/>
+      <c r="B45" s="1"/>
+      <c r="C45" s="1"/>
+      <c r="D45" s="3"/>
+      <c r="E45" s="3"/>
     </row>
     <row r="46" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D46" s="2"/>
-      <c r="E46" s="2"/>
+      <c r="A46" s="1"/>
+      <c r="B46" s="1"/>
+      <c r="C46" s="1"/>
+      <c r="D46" s="3"/>
+      <c r="E46" s="3"/>
     </row>
     <row r="47" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D47" s="2"/>
-      <c r="E47" s="2"/>
+      <c r="A47" s="1"/>
+      <c r="B47" s="1"/>
+      <c r="C47" s="1"/>
+      <c r="D47" s="3"/>
+      <c r="E47" s="3"/>
     </row>
     <row r="48" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D48" s="2"/>
-      <c r="E48" s="2"/>
+      <c r="A48" s="1"/>
+      <c r="B48" s="1"/>
+      <c r="D48" s="3"/>
+      <c r="E48" s="3"/>
     </row>
     <row r="49" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D49" s="2"/>
-      <c r="E49" s="2"/>
+      <c r="A49" s="1"/>
+      <c r="B49" s="1"/>
+      <c r="C49" s="1"/>
+      <c r="D49" s="3"/>
+      <c r="E49" s="3"/>
     </row>
     <row r="50" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D50" s="2"/>
-      <c r="E50" s="2"/>
+      <c r="A50" s="1"/>
+      <c r="B50" s="1"/>
+      <c r="C50" s="1"/>
+      <c r="D50" s="3"/>
+      <c r="E50" s="3"/>
     </row>
     <row r="51" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D51" s="2"/>
-      <c r="E51" s="2"/>
+      <c r="A51" s="1"/>
+      <c r="B51" s="1"/>
+      <c r="C51" s="1"/>
+      <c r="D51" s="3"/>
+      <c r="E51" s="3"/>
     </row>
     <row r="52" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D52" s="2"/>
-      <c r="E52" s="2"/>
+      <c r="A52" s="1"/>
+      <c r="B52" s="1"/>
+      <c r="C52" s="1"/>
+      <c r="D52" s="3"/>
+      <c r="E52" s="3"/>
     </row>
     <row r="53" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D53" s="2"/>
-      <c r="E53" s="2"/>
+      <c r="A53" s="1"/>
+      <c r="B53" s="1"/>
+      <c r="C53" s="1"/>
+      <c r="D53" s="3"/>
+      <c r="E53" s="3"/>
     </row>
     <row r="54" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D54" s="2"/>
-      <c r="E54" s="2"/>
+      <c r="A54" s="1"/>
+      <c r="B54" s="1"/>
+      <c r="C54" s="1"/>
+      <c r="D54" s="3"/>
+      <c r="E54" s="3"/>
     </row>
     <row r="55" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D55" s="2"/>
-      <c r="E55" s="2"/>
+      <c r="A55" s="1"/>
+      <c r="B55" s="1"/>
+      <c r="C55" s="1"/>
+      <c r="D55" s="3"/>
+      <c r="E55" s="3"/>
     </row>
     <row r="56" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D56" s="2"/>
-      <c r="E56" s="2"/>
+      <c r="A56" s="1"/>
+      <c r="B56" s="1"/>
+      <c r="C56" s="1"/>
+      <c r="D56" s="3"/>
+      <c r="E56" s="3"/>
     </row>
     <row r="57" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D57" s="2"/>

</xml_diff>